<commit_message>
Kit de Tareas Pastelería (ES LIVE): 09 con áreas de impresión y columna del resumen arregladas, y 02 C8 del merengue suizo, sin cambio de versión
Parche a nivel de XML (estilos, DV, CF, caché y docProps intactos), ronda 1 de la revisión de la edición EN:
- 09 «Instrucciones»: área de impresión A1:A20 → A1:B30 (el texto va en la B).
- 09 «Registro Mensual»: área A1:I38 → A1:J38 (entra «Responsable»).
- 09 «Cierre de Caja»: columna A 5 → 24 y B 50 → 31; los rótulos del Resumen de Cierre (A41-A46) ya no se parten.
- 02 «Cremas y Rellenos» C8: el merengue suizo no lleva almíbar → «Italiano: almíbar a 118-121 °C · suizo: claras y
  azúcar a 71 °C · mantequilla a 18-20 °C».
Volcado ES antes/después: solo esas 3 líneas (más los anchos). censo-entregables --fail 0 y gate-no-latinos 0.
Lo mismo en kit-pasteleria-v2_0-postprocess.py.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LzWqvTU1jPmLwXsDXHDGWJ
Via: Claude Code
</commit_message>
<xml_diff>
--- a/astro-site/public/dl/kit-tareas-pasteleria/09-apertura-cierre-caja.xlsx
+++ b/astro-site/public/dl/kit-tareas-pasteleria/09-apertura-cierre-caja.xlsx
@@ -13,13 +13,13 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Registro Mensual" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Instrucciones'!$A$1:$A$20</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Instrucciones'!$A$1:$B$30</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Apertura de Caja'!$4:$4</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="1">'Apertura de Caja'!$A$1:$F$18</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Cierre de Caja'!$4:$4</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="2">'Cierre de Caja'!$A$1:$F$48</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'Registro Mensual'!$4:$4</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="3">'Registro Mensual'!$A$1:$I$38</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="3">'Registro Mensual'!$A$1:$J$38</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1196,8 +1196,8 @@
   <dimension ref="A1:F50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="5" customWidth="1" min="1" max="1"/>
-    <col width="50" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="31" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>

</xml_diff>